<commit_message>
chore: fix repo name to be consistent identifier
</commit_message>
<xml_diff>
--- a/project/excel/common_domain_model.xlsx
+++ b/project/excel/common_domain_model.xlsx
@@ -5107,7 +5107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5118,20 +5118,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>identifer</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>messageInformation</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>party</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>partyRole</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>availableInventoryRecord</t>
         </is>
@@ -5153,82 +5163,102 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>expirationDateTime</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>collateral</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>partyRole</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>interestRate</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>dividendTerms</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>identifer</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet187.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>expirationDateTime</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>collateral</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
+          <t>availableInventoryType</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>identifer</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>messageInformation</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>partyRole</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>interestRate</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>identifer</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>security</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet187.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>availableInventoryType</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>messageInformation</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>partyRole</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>availableInventoryRecord</t>
         </is>

</xml_diff>